<commit_message>
W02 D1 decision workbook: the Start, Division, Average and Export tabs each open on the question the tab answers, and the Start tab says what each tab asks
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PqxrUdd3MVkcqi5tJL4ifU
</commit_message>
<xml_diff>
--- a/content/W02/D1/demos/C2_W02_D01_decision_tool_STUDENT.xlsx
+++ b/content/W02/D1/demos/C2_W02_D01_decision_tool_STUDENT.xlsx
@@ -490,7 +490,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The Monday numbers: the decision tool</t>
+          <t>Which four decisions stand behind the Retail-Plus line of Anand's sheet?</t>
         </is>
       </c>
     </row>
@@ -525,7 +525,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Customers: which count is a customer. Division: integers or numeric. Average: who is in the average. Sample: can the analyst rerun your five orders.</t>
+          <t>Customers asks which count is a customer. Division asks how often each segment's customers ordered, with the fraction kept. Average asks who is inside the average spend per member. Sample asks whether the analyst can rerun your five orders.</t>
         </is>
       </c>
     </row>
@@ -735,7 +735,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Integers or numeric?</t>
+          <t>How often did each segment's customers order, with the fraction kept?</t>
         </is>
       </c>
     </row>
@@ -1094,7 +1094,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Who is in the average?</t>
+          <t>Who is inside the average spend per Retail-Plus member?</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1521,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Anand's line, assembled</t>
+          <t>Is the Retail-Plus line ready for Anand's sheet?</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
W02 D1 day sheet, TA note and decision workbook after the reviews: the day sheet carries the fuller sentence to Anand, the renumbered close (S21 to S24, self-study D18 to D20 before it), every new key string, the 26 design items of 73, the guided build's minutes inside chapters 1 and 3, the new second routes and the companion's real path, and one-breath answers for all thirteen drill questions; the TA note splits its long opening, updates keys, debrief letters, hints and the drill; the workbook computes Division's change from the counts (Retail-Core 3.0 up) and its Sample tab sets Monday's unordered five against the rerun's, with no amount ties
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PqxrUdd3MVkcqi5tJL4ifU
</commit_message>
<xml_diff>
--- a/content/W02/D1/demos/C2_W02_D01_decision_tool_STUDENT.xlsx
+++ b/content/W02/D1/demos/C2_W02_D01_decision_tool_STUDENT.xlsx
@@ -561,7 +561,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Retail-Plus in Q2, counted three ways. Orders per customer is only as honest as the count under it.</t>
+          <t>Retail-Plus in Q2, counted three ways: the orders two ways and the customer table once. Orders per customer divides by whichever count you choose.</t>
         </is>
       </c>
     </row>
@@ -623,7 +623,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>members on the book</t>
+          <t>members on the customer table</t>
         </is>
       </c>
     </row>
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="B15" s="8">
-        <f>IF(ABS(ROUND(B12*B11,0)-B9)&gt;1,"Fix the ratio that divides by the wrong count before any number leaves the team.",IF(B10="order rows","Every member ordered exactly once: counting rows as customers erases the frequency branch.",IF(B10="members who bought","Retail-Plus, Q2: "&amp;B11&amp;" members bought, "&amp;TEXT(B12,"0.00")&amp;" orders each.","Retail-Plus, Q2: "&amp;TEXT(B12,"0.00")&amp;" orders per member on the book, which answers how often Kalpa's members order, whether or not they bought.")))</f>
+        <f>IF(ABS(ROUND(B12*B11,0)-B9)&gt;1,"Fix the ratio that divides by the wrong count before any number leaves the team.",IF(B10="order rows","Every member ordered exactly once: counting rows as customers erases the frequency branch.",IF(B10="members who bought","Retail-Plus, Q2: "&amp;B11&amp;" members bought, "&amp;TEXT(B12,"0.00")&amp;" orders each.","Retail-Plus, Q2: "&amp;TEXT(B12,"0.00")&amp;" orders per member on the customer table, which answers how often Kalpa's members order, whether or not they bought.")))</f>
         <v/>
       </c>
     </row>
@@ -708,7 +708,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"order rows,members who bought,members on the book"</formula1>
+      <formula1>"order rows,members who bought,members on the customer table"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1049,7 +1049,7 @@
         </is>
       </c>
       <c r="C20" s="8">
-        <f>IF(C14&gt;0,"Fix the honest column, which still drops the fraction, before reading any ratio.",C17&amp;" frequency moved from "&amp;TEXT(C18,"0.00")&amp;" to "&amp;TEXT(C19,"0.00")&amp;", "&amp;TEXT(ABS(C19/C18-1)*100,"0.0")&amp;" percent "&amp;IF(C19&lt;C18,"down","up")&amp;".")</f>
+        <f>IF(C14&gt;0,"Fix the honest column, which still drops the fraction, before reading any ratio.",C17&amp;" frequency moved from "&amp;TEXT(C18,"0.00")&amp;" to "&amp;TEXT(C19,"0.00")&amp;", "&amp;TEXT(ABS((SUMPRODUCT((A5:A12=C17)*(B5:B12="Q2")*C5:C12)/SUMPRODUCT((A5:A12=C17)*(B5:B12="Q2")*D5:D12))/(SUMPRODUCT((A5:A12=C17)*(B5:B12="Q1")*C5:C12)/SUMPRODUCT((A5:A12=C17)*(B5:B12="Q1")*D5:D12))-1)*100,"0.0")&amp;" percent "&amp;IF(C19&lt;C18,"down","up")&amp;".")</f>
         <v/>
       </c>
     </row>
@@ -1278,7 +1278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1299,19 +1299,19 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>The first eight delivered Q2 app orders by order id. A sample is reproducible only when its order is unique.</t>
+          <t>Five delivered Q2 app orders drawn with LIMIT 5 and no ORDER BY, on Monday and after the overnight reload rewrote two rows with their own values.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>order_id</t>
+          <t>Monday, no ORDER BY</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>amount (Rs)</t>
+          <t>After the reload, no ORDER BY</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -1321,7 +1321,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Unique in this table?</t>
+          <t>Repeatable?</t>
         </is>
       </c>
     </row>
@@ -1331,8 +1331,10 @@
           <t>KR-00542</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>790</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>KR-00545</t>
+        </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1341,7 +1343,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -1351,12 +1353,14 @@
           <t>KR-00544</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>960</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>KR-00546</t>
+        </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>amount</t>
+          <t>order_id</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1371,17 +1375,9 @@
           <t>KR-00545</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>680</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>order_id</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>yes</t>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>KR-00547</t>
         </is>
       </c>
     </row>
@@ -1391,8 +1387,10 @@
           <t>KR-00546</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>500</v>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>KR-00549</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -1401,100 +1399,72 @@
           <t>KR-00547</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>970</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>KR-00549</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>970</v>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>KR-00553</t>
+        </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>KR-00553</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>1470</v>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Your ORDER BY</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>order_id</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>KR-00555</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>770</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Your ORDER BY</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>order_id</t>
-        </is>
+          <t>Monday's orders the rerun drew again</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>SUMPRODUCT(COUNTIF(B5:B9,A5:A9))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>The check</t>
+        </is>
+      </c>
+      <c r="B13" s="2">
+        <f>IF(AND(E5="yes",B12&lt;5),"The table calls no ORDER BY repeatable, and the rerun after the reload drew "&amp;B12&amp;" of Monday's five. Fix it first.","The repeatable column matches the two runs.")</f>
+        <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Amounts shared by two orders</t>
-        </is>
-      </c>
-      <c r="B15">
-        <f>SUMPRODUCT((COUNTIF(B5:B12,B5:B12)&gt;1)*1)</f>
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="B15" s="8">
+        <f>IF(AND(E5="yes",B12&lt;5),"Fix the repeatable column before choosing an order.",IF(INDEX(E5:E6,MATCH(B11,D5:D6,0))="yes","Order by "&amp;B11&amp;", then LIMIT 5: the analyst gets the same five orders on every run.","With no ORDER BY the five can change between runs, as the reload showed, so the analyst may trace a different five."))</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>The check</t>
-        </is>
-      </c>
-      <c r="B16" s="2">
-        <f>IF(AND(E6="yes",B15&gt;0),"The table calls amount unique, and "&amp;B15&amp;" orders share an amount. Fix it first.","The uniqueness column matches the data.")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>Verdict</t>
-        </is>
-      </c>
-      <c r="B18" s="8">
-        <f>IF(AND(E6="yes",B15&gt;0),"Fix the uniqueness column before choosing an order.",IF(INDEX(E5:E7,MATCH(B14,D5:D7,0))="yes","Order by "&amp;B14&amp;", then LIMIT 5: the analyst gets the same five orders on every run.","Ordering by "&amp;B14&amp;" leaves the five free to change between runs, so the audit cannot be repeated."))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Fixed, for the Export tab</t>
         </is>
       </c>
-      <c r="B19">
-        <f>IF(AND(E6="yes",B15&gt;0),0,IF(INDEX(E5:E7,MATCH(B14,D5:D7,0))="yes",1,0))</f>
+      <c r="B16">
+        <f>IF(AND(E5="yes",B12&lt;5),0,IF(INDEX(E5:E6,MATCH(B11,D5:D6,0))="yes",1,0))</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"nothing,amount,order_id"</formula1>
+    <dataValidation sqref="B11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"nothing,order_id"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1539,7 +1509,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>Customers!B16+Division!C21+Average!B18+Sample!B19</f>
+        <f>Customers!B16+Division!C21+Average!B18+Sample!B16</f>
         <v/>
       </c>
     </row>
@@ -1561,7 +1531,7 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <f>IF(B4=4,"Customers: "&amp;Customers!B15&amp;CHAR(10)&amp;"Frequency: "&amp;Division!C20&amp;CHAR(10)&amp;"Spend: "&amp;Average!B17&amp;CHAR(10)&amp;"Audit: "&amp;Sample!B18,"The line assembles once every tab passes its check.")</f>
+        <f>IF(B4=4,"Customers: "&amp;Customers!B15&amp;CHAR(10)&amp;"Frequency: "&amp;Division!C20&amp;CHAR(10)&amp;"Spend: "&amp;Average!B17&amp;CHAR(10)&amp;"Audit: "&amp;Sample!B15,"The line assembles once every tab passes its check.")</f>
         <v/>
       </c>
     </row>

</xml_diff>